<commit_message>
Stabilize oxygen runtime for surfacing
</commit_message>
<xml_diff>
--- a/mod-here/LongSubmerged10x/Data Sheets/General.xlsx
+++ b/mod-here/LongSubmerged10x/Data Sheets/General.xlsx
@@ -89,13 +89,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45.54296875" customWidth="1" min="1" max="1"/>
@@ -541,28 +540,6 @@
         <v>-1.333333333333333e-05</v>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>/Resources</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Oxygen Consumption Per Character</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>-5e-09</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>